<commit_message>
Add API testing sprint2 scripts for user management , traffic logs and export log
</commit_message>
<xml_diff>
--- a/test/ApiTesting.xlsx
+++ b/test/ApiTesting.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Software Engineering\PaiNamNaeWebAppSec2_6\test\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{748961BE-4908-4562-AF70-25E0ACA7446C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99F2C70E-A757-4849-8838-69C5CAFE8A22}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{07978156-2A2C-42E9-A898-AA58910779AE}"/>
   </bookViews>
@@ -349,22 +349,46 @@
   </cellStyleXfs>
   <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -372,30 +396,6 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -743,170 +743,170 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="22.8">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="14" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="2"/>
-      <c r="C1" s="2"/>
-      <c r="D1" s="2"/>
-      <c r="E1" s="2"/>
-      <c r="F1" s="3"/>
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="11"/>
     </row>
     <row r="2" spans="1:6" ht="22.8">
-      <c r="A2" s="4"/>
-      <c r="B2" s="4"/>
-      <c r="C2" s="4"/>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
-      <c r="F2" s="4"/>
+      <c r="A2" s="1"/>
+      <c r="B2" s="1"/>
+      <c r="C2" s="1"/>
+      <c r="D2" s="1"/>
+      <c r="E2" s="1"/>
+      <c r="F2" s="1"/>
     </row>
     <row r="3" spans="1:6" ht="22.8">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="2"/>
-      <c r="D3" s="5" t="s">
+      <c r="C3" s="13"/>
+      <c r="D3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="E3" s="7"/>
-      <c r="F3" s="3"/>
+      <c r="E3" s="12"/>
+      <c r="F3" s="11"/>
     </row>
     <row r="4" spans="1:6" ht="22.8">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="8"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="5" t="s">
+      <c r="B4" s="16"/>
+      <c r="C4" s="13"/>
+      <c r="D4" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="E4" s="9"/>
-      <c r="F4" s="3"/>
+      <c r="E4" s="17"/>
+      <c r="F4" s="11"/>
     </row>
     <row r="5" spans="1:6" ht="22.8">
-      <c r="A5" s="5" t="s">
+      <c r="A5" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="7"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="5" t="s">
+      <c r="B5" s="12"/>
+      <c r="C5" s="13"/>
+      <c r="D5" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="E5" s="10"/>
-      <c r="F5" s="3"/>
+      <c r="E5" s="18"/>
+      <c r="F5" s="11"/>
     </row>
     <row r="6" spans="1:6" ht="22.8">
-      <c r="A6" s="11" t="s">
+      <c r="A6" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="3"/>
-      <c r="C6" s="7"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="3"/>
+      <c r="B6" s="11"/>
+      <c r="C6" s="12"/>
+      <c r="D6" s="13"/>
+      <c r="E6" s="13"/>
+      <c r="F6" s="11"/>
     </row>
     <row r="7" spans="1:6" ht="22.8">
-      <c r="A7" s="4"/>
-      <c r="B7" s="4"/>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-      <c r="E7" s="4"/>
-      <c r="F7" s="4"/>
+      <c r="A7" s="1"/>
+      <c r="B7" s="1"/>
+      <c r="C7" s="1"/>
+      <c r="D7" s="1"/>
+      <c r="E7" s="1"/>
+      <c r="F7" s="1"/>
     </row>
     <row r="8" spans="1:6" ht="17.399999999999999">
-      <c r="A8" s="12" t="s">
+      <c r="A8" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B8" s="12" t="s">
+      <c r="B8" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="12" t="s">
+      <c r="C8" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="D8" s="16" t="s">
+      <c r="D8" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E8" s="12" t="s">
+      <c r="E8" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="F8" s="12" t="s">
+      <c r="F8" s="3" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:6" ht="133.19999999999999" customHeight="1">
-      <c r="A9" s="13" t="s">
+      <c r="A9" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="18" t="s">
+      <c r="B9" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="C9" s="17" t="s">
+      <c r="C9" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="D9" s="17" t="s">
+      <c r="D9" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="E9" s="17" t="s">
+      <c r="E9" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="F9" s="18">
+      <c r="F9" s="7">
         <v>201</v>
       </c>
     </row>
     <row r="10" spans="1:6" ht="124.2">
-      <c r="A10" s="14"/>
-      <c r="B10" s="18" t="s">
+      <c r="A10" s="9"/>
+      <c r="B10" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="C10" s="17" t="s">
+      <c r="C10" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="D10" s="17" t="s">
+      <c r="D10" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="E10" s="17" t="s">
+      <c r="E10" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="F10" s="18">
+      <c r="F10" s="7">
         <v>200</v>
       </c>
     </row>
     <row r="11" spans="1:6" ht="111" customHeight="1">
-      <c r="A11" s="14"/>
-      <c r="B11" s="18" t="s">
+      <c r="A11" s="9"/>
+      <c r="B11" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="C11" s="15" t="s">
+      <c r="C11" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D11" s="17" t="s">
+      <c r="D11" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="E11" s="17" t="s">
+      <c r="E11" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="F11" s="18">
+      <c r="F11" s="7">
         <v>200</v>
       </c>
     </row>
     <row r="12" spans="1:6" ht="55.2">
-      <c r="A12" s="14"/>
-      <c r="B12" s="18" t="s">
+      <c r="A12" s="9"/>
+      <c r="B12" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="C12" s="17" t="s">
+      <c r="C12" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="D12" s="17" t="s">
+      <c r="D12" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="E12" s="17" t="s">
+      <c r="E12" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="F12" s="18">
+      <c r="F12" s="7">
         <v>404</v>
       </c>
     </row>

</xml_diff>